<commit_message>
Actualizaciones garndes antes de la publicación en línea.
</commit_message>
<xml_diff>
--- a/baseline/alumnos.xlsx
+++ b/baseline/alumnos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiriosr/Projects/www/classManager/baseline/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiriosr/Projects/www/class_manager/baseline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA960A6-EE0D-2943-9C43-34F50910EBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDAF97DF-8AB5-CE46-B97F-3200D141AA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16660" xr2:uid="{642C14C2-41B4-0A42-B2DB-5DF7F625DFAA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="45">
   <si>
     <t> CAMPOS MORALES ALINE CAROLINA</t>
   </si>
@@ -144,13 +144,43 @@
   </si>
   <si>
     <t>VAZQUEZ LARA MARIA GUADALUPE</t>
+  </si>
+  <si>
+    <t>Carrera</t>
+  </si>
+  <si>
+    <t>Ingeniería en Tecnología Ambiental</t>
+  </si>
+  <si>
+    <t>Ingeniería en Energías Renovables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grupo </t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Cuatrimestre</t>
+  </si>
+  <si>
+    <t>Ciclo</t>
+  </si>
+  <si>
+    <t>Materia</t>
+  </si>
+  <si>
+    <t>Inglés VIII</t>
+  </si>
+  <si>
+    <t>26C1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -163,6 +193,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -529,285 +565,797 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90156616-E2FA-8345-818F-CA7F25F06525}">
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>612310471</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>612310140</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>612310554</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>612310481</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>612310607</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>612310189</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>612310405</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>612310450</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>612310131</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>612310432</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>612310161</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>612310576</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>612310574</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>612310503</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>612310220</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>612310550</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>612310216</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18">
+        <v>8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>612310272</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>612310173</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>612310273</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>612310545</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22">
+        <v>8</v>
+      </c>
+      <c r="F22" t="s">
+        <v>44</v>
+      </c>
+      <c r="G22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>612310128</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23">
+        <v>8</v>
+      </c>
+      <c r="F23" t="s">
+        <v>44</v>
+      </c>
+      <c r="G23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>612310647</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24">
+        <v>8</v>
+      </c>
+      <c r="F24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>612110492</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25">
+        <v>8</v>
+      </c>
+      <c r="F25" t="s">
+        <v>44</v>
+      </c>
+      <c r="G25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>612310552</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C26" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26">
+        <v>8</v>
+      </c>
+      <c r="F26" t="s">
+        <v>44</v>
+      </c>
+      <c r="G26" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>612310252</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C27" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27">
+        <v>8</v>
+      </c>
+      <c r="F27" t="s">
+        <v>44</v>
+      </c>
+      <c r="G27" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>612310114</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C28" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>44</v>
+      </c>
+      <c r="G28" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>612310335</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" t="s">
+        <v>39</v>
+      </c>
+      <c r="E29">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>44</v>
+      </c>
+      <c r="G29" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>612310083</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30">
+        <v>8</v>
+      </c>
+      <c r="F30" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>612310556</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" t="s">
+        <v>39</v>
+      </c>
+      <c r="E31">
+        <v>8</v>
+      </c>
+      <c r="F31" t="s">
+        <v>44</v>
+      </c>
+      <c r="G31" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>612310171</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32">
+        <v>8</v>
+      </c>
+      <c r="F32" t="s">
+        <v>44</v>
+      </c>
+      <c r="G32" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>612310518</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C33" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>44</v>
+      </c>
+      <c r="G33" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>612210579</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="C34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" t="s">
+        <v>39</v>
+      </c>
+      <c r="E34">
+        <v>8</v>
+      </c>
+      <c r="F34" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" t="s">
+        <v>43</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>